<commit_message>
Close BOMs (#40): wire up khbomvariant, rebuild deliverables package, refresh reports
Adds build_boms()/build_bom_combined() in transform_odoo.py, extracting the newly
self-service-published khbomvariant OData service (400 headers, 448 variants, 14,948
component lines) into mrp_bom.csv / mrp_bom_line.csv / mrp_bom_with_lines.csv. Registry
flips #40 from pending_mapping to built, leaving Equipment (#34) as the only open
mandatory object.

Deliverables package gains file #20 (BOM header+lines combined, all three folders plus
custom-field checklist rows), README updated to match. diagnostics/validate_masters.py
now checks mrp_bom.csv/mrp_bom_line.csv. PROJECT_STATUS.csv, CONSOLIDATED_STATUS.csv,
SAP_Field_Mapping.xlsx, and the diagnostics reports are regenerated against current disk
state. sap_odata_editor_walkthrough/ documents the OData Editor build process with
screenshots.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SAP_Field_Mapping.xlsx
+++ b/SAP_Field_Mapping.xlsx
@@ -2168,9 +2168,9 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>pending_mapping</t>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>built</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -13032,7 +13032,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>REAL DATA: same khlocation source as #28, filtered on InventoryManagedLocationIndicator (ByDesign's own signal for 'this location tracks inventory') - 1/4 locations qualify</t>
+          <t>REAL DATA: same khlocation source as #28, filtered on InventoryManagedLocationIndicator (ByDesign's own signal for 'this location tracks inventory') - 1/1 locations qualify as of 2026-09-25 (tenant used to have 4 sites; confirmed live it now has only 1, 'Danlaw Technologies India Limited' - a tenant-side change, not a pipeline gap)</t>
         </is>
       </c>
     </row>
@@ -13924,7 +13924,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>REAL DATA: khlocation custom service, 4 locations</t>
+          <t>REAL DATA: khlocation custom service, 1 site as of 2026-09-25 (was 4; confirmed live - see #27 note) plus its storage areas</t>
         </is>
       </c>
     </row>
@@ -19312,10 +19312,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19328,24 +19333,1125 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Module: Manufacturing  |  Category: Master  |  Mandatory: Yes  |  Odoo model: mrp.bom  |  Status: PENDING_MAPPING</t>
+          <t>Module: Manufacturing  |  Category: Master  |  Mandatory: Yes  |  Odoo model: mrp.bom  |  Status: BUILT</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>NOT OBTAINABLE OVER ODATA FROM THIS TENANT - the strongest negative result in the project, and the one mandatory object that genuinely cannot be closed from here. Searched for bom / 'bill of material' / 'production model' / recipe / component / routing / explosion across BOTH (a) all 1485 entity sets of all 48 services the tenant publishes to this user (schema_snapshots/service_catalog.json, SERVICE_CATALOG.csv) and (b) all 609 entity sets defined across all 47 custom service .xml files - zero matches in either. Importing more custom services cannot produce it: no BOM service definition exists in the sample set. The design-time catalog does list PBOM data sources (SCMPBOMU02 etc), but they are NOT published as OData on this tenant - that catalog tracks report definitions, not published services. khproductionorder REFERENCES a BOM via ProductionModelID/ProductionModelVersionID but never exposes its components. Options for the user: expose the PBOM data sources via Business Configuration &gt; Analytics, or extract BOMs by a non-OData route (UI export / file download) and hand over a CSV.</t>
+          <t>REAL DATA, closed 2026-09-25. Confirmed unobtainable via the tenant's 1485 built-in + 609 custom-.xml entity sets (an exhaustive negative result, still true of THAT set) - but the data itself was real, visible live in the ByDesign UI under Enterprise Search &gt; 'Bills of Material Variants'. Closed by building a brand new custom OData service (khbomvariant) directly via the OData Editor - self-service, no .xml import needed - exposing the underlying ProductionBillOfMaterial standard Business Object for the first time. 400 BOM headers, 448 variants (447 non-obsolete -&gt; mrp_bom.csv rows), 14,947 component lines -&gt; mrp_bom_line.csv. product_tmpl_id/id and each line's product_id/id resolve via the same MaterialUUID -&gt; InternalID lookup used for product_template.csv (1/447 boms and 0/14947 lines unresolved). Verified against the live UI screen for one real BOM (CS90861DOOO): all 5 components shown on screen matched exactly (products + quantities), plus 8 more from other item groups not visible in that screen's scroll position. Known limitation: components attach to the BOM header, not a specific variant, so the 48 headers with multiple variants get the same component list per variant - matches what the raw data actually supports. Full story + screenshots: sap_odata_editor_walkthrough/bom_service_setup/README.md.</t>
         </is>
       </c>
     </row>
     <row r="4"/>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>No SAP data extracted yet for this object - see the notes above and CLAUDE.md.</t>
-        </is>
-      </c>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>SAP Entity (raw source)</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>SAP Field Name</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Sample Value</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Mapped Odoo Field</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Target Odoo Model</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialCollection</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>PCBA FOR GEAR MOTOR</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialCollection</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>BGMBETTCARD7</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialCollection</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>LogisticsPreparationFunctionalUnitID</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialCollection</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>LogisticsPreparationFunctionalUnitUUID</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialCollection</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>ObjectID</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>00163E5F7A721ED9898C36894601C402</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>(join key)</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Header - looked up by ProductionBillOfMaterialVariantCollection.ParentObjectID</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialCollection</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>UUID</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>00163E5F-7A72-1ED9-898C-36894601C402</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialVariantCollection</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Variant's own ID; mrp_bom.csv's code uses the header's ID instead</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialVariantCollection</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>MaterialUUID</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>00163E5F-7A72-1ED9-88DC-8CE74D155AE0</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>product_tmpl_id/id</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Via the same MaterialUUID -&gt; InternalID lookup used for product_template.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialVariantCollection</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>ObjectID</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>00163E5F7A721ED9898C368946022402</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>id (external ID key)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialVariantCollection</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>ObsoleteIndicator</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>(filter only, not mapped)</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete variants (1/448) excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialVariantCollection</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>ParentObjectID</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>00163E5F7A721ED9898C36894601C402</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>(join key)</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>-&gt; ProductionBillOfMaterialCollection.ObjectID</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialVariantCollection</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>1.00000000000000</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>product_qty</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialVariantCollection</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>unitCode</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>ZNO</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupCollection</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>BillOfMaterialID</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>BGMBETTCARD7</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>(not used, not mapped)</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupCollection</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>BillOfMaterialItemGroupID</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>(not used, not mapped)</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupCollection</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>(not used, not mapped)</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupCollection</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>ItemRequiredIndicator</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr"/>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>(not used, not mapped)</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupCollection</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>MultipleSelectionAllowedIndicator</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>(not used, not mapped)</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupCollection</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>ObjectID</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>00163E5F7A721ED9898C368946028402</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>(not used, not mapped)</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Raw-extracted but not used - this entity is a thin pointer node with no component data of its own and a broken $expand back to its parent on this tenant; see build_boms() docstring. Real component data comes from ItemGroupItemChangeStateCollection instead</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupCollection</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>ParentObjectID</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>00163E5F7A721ED9898C36894601C402</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>(not used, not mapped)</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupCollection</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>UUID</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>00163E5F-7A72-1ED9-898C-368946028402</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>(not used, not mapped)</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>DeletedIndicator</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>(filter only, not mapped)</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Deleted component lines excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>EngineeringChangeOrderID</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>BGMBETTCARD7</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>MaterialUUID</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>00163E5F-7A72-1ED9-88DC-8CE74D157AE0</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>product_id/id</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Component product, via the same MaterialUUID -&gt; InternalID lookup</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>ObjectID</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>00163E5F7A721ED9898C368946036402</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>(part of id)</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Combined with the variant's ObjectID to form mrp_bom_line.csv's external id</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterial.Description</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>PCBA FOR GEAR MOTOR</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>$expand artifact</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterial.ID</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>BGMBETTCARD7</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>$expand artifact</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterial.LogisticsPreparationFunctionalUnitID</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr"/>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>$expand artifact</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterial.LogisticsPreparationFunctionalUnitUUID</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr"/>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>$expand artifact</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterial.ObjectID</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>00163E5F7A721ED9898C36894601C402</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>(join key)</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Populated via $expand=ProductionBillOfMaterial - the real BOM header link (ItemGroupItemCollection's own nav property back to its parent is broken on this tenant, see build_boms() docstring)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterial.UUID</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>00163E5F-7A72-1ED9-898C-36894601C402</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>$expand artifact</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>1.00000000000000</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>product_qty</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>QuantityFixedIndicator</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>UUID</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>00163E5F-7A72-1ED9-898C-368946036402</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>__metadata.type</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>cust.ProductionBillOfMaterialItemGroupItemChangeState</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>(technical, not mapped)</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>__metadata.uri</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>https://my346623.sapbydesign.com/sap/byd/odata/cust/v1/khbom...</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>(technical, not mapped)</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>ProductionBillOfMaterialItemGroupItemChangeStateCollection</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>unitCode</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>ZNO</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>mrp.bom.line</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19432,7 +20538,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>REAL DATA: derived from khproductionorder's OperationCollection (ResourceID/ResourceDescription), deduplicated - no dedicated Work Center master service found, but this data was already on hand (used for #44) - 18 distinct work centers</t>
+          <t>REAL DATA: derived from khproductionorder's OperationCollection (ResourceID/ResourceDescription), deduplicated - no dedicated Work Center master service found, but this data was already on hand (used for #44) - 17 distinct work centers as of 2026-09-25 (was 18 earlier - minor drift in the source data, negligible)</t>
         </is>
       </c>
     </row>
@@ -37964,7 +39070,11 @@
           <t>BankGroupCode</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr"/>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
           <t>(not mapped)</t>
@@ -37988,7 +39098,11 @@
           <t>BankGroupCodeText</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr"/>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Corporation Bank</t>
+        </is>
+      </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
           <t>(not mapped)</t>
@@ -38068,7 +39182,11 @@
           <t>CommonBankStandardIDMainIndicator</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
           <t>(not mapped)</t>
@@ -38148,7 +39266,11 @@
           <t>DeletedIndicator</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr"/>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
           <t>(not mapped)</t>
@@ -38284,7 +39406,11 @@
           <t>RegionCode</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr"/>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
           <t>(not mapped)</t>
@@ -38308,7 +39434,11 @@
           <t>RegionCodeText</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr"/>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Goa</t>
+        </is>
+      </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
           <t>(not mapped)</t>
@@ -38332,7 +39462,11 @@
           <t>StreetName</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr"/>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Collyer Quay Branch</t>
+        </is>
+      </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
           <t>(not mapped)</t>
@@ -39468,7 +40602,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>REAL DATA: khsalesarrangement custom service, 35 arrangements. partner_id/id NOT populated - CustomerUUID here is a hyphenated GUID that doesn't match res_partner's numeric-ID-based external IDs, and this tenant hasn't exposed a UUID-&gt;numeric-ID lookup</t>
+          <t>REAL DATA: 226 pricelists, one per real SAP Sales Arrangement resolved from khsalesorder via _resolve_order_to_arrangement() (Customer + SalesOrg + DistributionChannel business key) - not one synthetic catch-all. partner_id/id NOT populated - CustomerUUID here is a hyphenated GUID that doesn't match res_partner's numeric-ID-based external IDs, and this tenant hasn't exposed a UUID-&gt;numeric-ID lookup</t>
         </is>
       </c>
     </row>
@@ -40192,7 +41326,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>THIS TENANT HAS NO DISCOUNT RULES - checked, not assumed: of the 94 price components SAP categorises as 'Discount', every non-zero one is a Rounding Difference, and Item Discounts / Header Discounts are 0.00 throughout. Nothing was invented to fill the gap. What the same price-component data does carry is real LIST PRICES (269 components typed 'List Price', 97 distinct values), and product.pricelist.item is Odoo's model for 'this product is priced at X' - so this file holds 41 price rules under a dedicated 'SAP List Prices' pricelist, kept separate from the sales arrangements written for #59. Where a product was quoted at several prices the most frequent wins; the full per-order history is in output_full_csv/.</t>
+          <t>THIS TENANT HAS NO DISCOUNT RULES - checked, not assumed: of the 94 price components SAP categorises as 'Discount', every non-zero one is a Rounding Difference, and Item Discounts / Header Discounts are 0.00 throughout. Nothing was invented to fill the gap. What the same price-component data does carry is real LIST PRICES, and product.pricelist.item is Odoo's model for 'this product is priced at X' - so this file holds 1109 price lines attached to their real resolved #59 pricelists (61 of 226 carry lines); only the 8 orders whose Sales Arrangement couldn't be resolved fall into a small 'SAP List Prices - Unmatched Sales Arrangement' fallback pricelist. Where a product was quoted at several prices the most frequent wins; the full per-order history is in output_full_csv/.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close Equipment (#34): wire up khequipmentresource, closing every mandatory object
Adds build_equipment() in transform_odoo.py, extracting the newly self-service-published
khequipmentresource OData service (18 Equipment Resources, real ByDesign standard master
data under "Supply Chain Design Master Data" -> "Resources") into maintenance_equipment.csv.
Registry flips #34 from not_in_bydesign to built - every mandatory sheet object now has a
real SAP source.

Deliverables package gains file #21 (equipment, all three folders plus custom-field
checklist rows), both READMEs updated. diagnostics/validate_masters.py now checks
maintenance_equipment.csv. export_full_csv.py gains a MODEL_ROOTS/ODOO_KEY entry so the
full-column export enriches it with sap__khequipmentresource__... columns.
PROJECT_STATUS.csv, CONSOLIDATED_STATUS.csv, SAP_Field_Mapping.xlsx, and the diagnostics
reports are regenerated against current disk state.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SAP_Field_Mapping.xlsx
+++ b/SAP_Field_Mapping.xlsx
@@ -1928,9 +1928,9 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>not_in_bydesign</t>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>built</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -12628,7 +12628,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>REAL DATA: khopportunity custom service, 15 opportunities (all, unfiltered)</t>
+          <t>khopportunity custom service - transform code is real and correct, but confirmed live on 2026-09-26 (direct curl, $inlinecount=allpages) that OpportunityCollection currently has 0 rows on this tenant - down from the 15 this note previously described. Not a pipeline bug: crm_lead.csv/_open/_closed are correctly empty because the source data is currently empty. Re-check live if this matters before go-live; the code will pick up real rows automatically the moment the tenant has any.</t>
         </is>
       </c>
     </row>
@@ -12704,7 +12704,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>REAL DATA: same khopportunity source as #20, filtered on LifeCycleStatusCode (Open=1, In Process=2) - 8/15 open</t>
+          <t>Same khopportunity source and same currently-empty-tenant caveat as #20 (filter logic: LifeCycleStatusCode Open=1/In Process=2, confirmed correct in code, just has nothing to filter right now).</t>
         </is>
       </c>
     </row>
@@ -12780,7 +12780,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>REAL DATA: same khopportunity source as #20, filtered on LifeCycleStatusCode (Won=4, Lost=5) - 7/15 closed</t>
+          <t>Same khopportunity source and same currently-empty-tenant caveat as #20 (filter logic: LifeCycleStatusCode Won=4/Lost=5, confirmed correct in code, just has nothing to filter right now).</t>
         </is>
       </c>
     </row>
@@ -19010,10 +19010,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19026,22 +19031,387 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Module: Maintenance  |  Category: Master  |  Mandatory: Yes  |  Odoo model: maintenance.equipment  |  Status: NOT_IN_BYDESIGN</t>
+          <t>Module: Maintenance  |  Category: Master  |  Mandatory: Yes  |  Odoo model: maintenance.equipment  |  Status: BUILT</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>MANDATORY - investigated twice. (1) Zero matches for 'equipment' across the tenant's 573-entry Design Data Sources catalog. (2) User imported+tested tmserviceorder/tmserviceconfirmation/tmservicerequest (Service Order/Confirmation/Request custom services) as a possible alternate path: their metadata confirms NO standalone Equipment entity exists in any of them - ReferenceObjectCollection only carries ProductID(+SerialID), i.e. ByDesign models 'equipment' as a serialized Product instance, not separate master data. tmserviceorder/tmservicerequest data access is additionally blocked by SAP authorization restrictions for the SDK user (metadata visible, data reads return RBAM_ERROR); tmserviceconfirmation is accessible but has 0 rows on this tenant. CONCLUSION: standard ByDesign has no Equipment master data object - if this data is needed, it must come from a different source system or be confirmed out of scope with Danlaw/the client.</t>
+          <t>MANDATORY - closed 2026-09-28. Earlier notes (kept for context) correctly found no standalone 'Equipment' master data object in any standard or custom service - ByDesign genuinely has no Preventive Maintenance module. What resolves the sheet requirement instead: the real ByDesign standard Business Object EquipmentResource ('Supply Chain Design Master Data' -&gt; 'Resources' in the live UI, the same discovery as khbomvariant) - 18 real records (SMT lines, wave soldering, final inspection, etc.), genuinely typed 'Equipment Resource' on this tenant. Never published as OData until built directly via the OData Editor (self-service, no .xml import): service khequipmentresource, Work Center View SCM_RESOURCES (found by searching the picker for 'Resources' - it only matches a Work Center View's own display name, not its technical ID or parent Work Center name, which is why 'Equipment'/'Design'/'Master Data' searches all returned zero results first). See build_equipment() in src/transform_odoo.py; raw_sources below.</t>
         </is>
       </c>
     </row>
     <row r="4"/>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>No SAP data extracted yet for this object - see the notes above and CLAUDE.md.</t>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>SAP Entity (raw source)</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>SAP Field Name</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Sample Value</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Mapped Odoo Field</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Target Odoo Model</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>EquipmentResourceCollection</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>CategoryCode</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>maintenance.equipment</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>EquipmentResourceCollection</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>SMT LINES WITH PRINTER, SPI, PLACEMENT &amp;</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>maintenance.equipment</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>EquipmentResourceCollection</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>FinancialRelevanceIndicator</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>maintenance.equipment</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>EquipmentResourceCollection</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>10100</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>serial_no</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>maintenance.equipment</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>The resource's own business ID, e.g. "10100"</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>EquipmentResourceCollection</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>ObjectID</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>00163E5F7A721EE989AE67C5DD490CF0</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>id (external ID key)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>maintenance.equipment</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>EquipmentResourceCollection</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>ProductionSchedulingRelevanceIndicator</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>maintenance.equipment</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>EquipmentResourceCollection</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>ResourceMultipleIndicator</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>maintenance.equipment</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>EquipmentResourceCollection</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>ResourceTimeZoneCode</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>INDIA</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>maintenance.equipment</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>EquipmentResourceCollection</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>SupplyPlanningRelevanceIndicator</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>maintenance.equipment</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>EquipmentResourceCollection</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>UUID</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>00163E5F-7A72-1EE9-89AE-67C5DD490CF0</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>maintenance.equipment</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>EquipmentResourceCollection</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>WorkingDayCalendarCode</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Z98Z</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>(no core Odoo field)</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>maintenance.equipment</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>EquipmentResourceCollection</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>languageCode</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>(filter only)</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>maintenance.equipment</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Always EN on this tenant</t>
         </is>
       </c>
     </row>
@@ -43083,7 +43453,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>khcustomerquote custom service is imported and live (metadata confirmed, CustomerQuoteCollection has real fields) but data reads are blocked by SAP authorization restrictions for the SDK user (RBAM_ERROR) - needs broader permissions granted on this tenant before it can be extracted</t>
+          <t>UPDATED 2026-09-26: the authorization block described here is resolved - live curl now returns HTTP 200 with $inlinecount __count=0 (not RBAM_ERROR). khcustomerquote is imported, live, and authorized; the tenant genuinely just has zero customer quotes right now. Still pending_mapping because there's no data to confirm a transform against, not because of access - re-check if the tenant gets real quote data later.</t>
         </is>
       </c>
     </row>

</xml_diff>